<commit_message>
Cambios en Catalogo maestro
</commit_message>
<xml_diff>
--- a/database/catalogos/catalogo_maestro.xlsx
+++ b/database/catalogos/catalogo_maestro.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1193" uniqueCount="604">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1205" uniqueCount="609">
   <si>
     <t>slug</t>
   </si>
@@ -439,16 +439,10 @@
     <t>Desechable grande</t>
   </si>
   <si>
-    <t>pozole_chico</t>
-  </si>
-  <si>
-    <t>Pozole chico</t>
-  </si>
-  <si>
-    <t>pozole_grande</t>
-  </si>
-  <si>
-    <t>Pozole grande</t>
+    <t>pozole</t>
+  </si>
+  <si>
+    <t>Pozole</t>
   </si>
   <si>
     <t>otro</t>
@@ -823,6 +817,12 @@
     <t>Bebida del paquete</t>
   </si>
   <si>
+    <t>tamano_pozole</t>
+  </si>
+  <si>
+    <t>Tamano Pozole</t>
+  </si>
+  <si>
     <t>proteina_pozole</t>
   </si>
   <si>
@@ -1552,6 +1552,24 @@
     <t>Bebida del paquete: Te</t>
   </si>
   <si>
+    <t>tamano_pozole_chico</t>
+  </si>
+  <si>
+    <t>Tamano Pozole: Chico</t>
+  </si>
+  <si>
+    <t>Pozole Grande</t>
+  </si>
+  <si>
+    <t>tamano_pozole_grande</t>
+  </si>
+  <si>
+    <t>Tamano Pozole: Grande</t>
+  </si>
+  <si>
+    <t>Pozole Chico</t>
+  </si>
+  <si>
     <t>proteina_pozole_sin_proteina</t>
   </si>
   <si>
@@ -1765,10 +1783,7 @@
     <t>DESECHABLE GRANDE</t>
   </si>
   <si>
-    <t>POZOLE CHICO</t>
-  </si>
-  <si>
-    <t>POZOLE GRANDE</t>
+    <t>POZOLE</t>
   </si>
   <si>
     <t>fecha</t>
@@ -5944,7 +5959,7 @@
       <c r="G53" s="2">
         <v>1.0</v>
       </c>
-      <c r="H53" s="2">
+      <c r="H53" s="4">
         <v>0.0</v>
       </c>
       <c r="I53" s="2">
@@ -5983,10 +5998,10 @@
         <v>13</v>
       </c>
       <c r="D54" s="4">
-        <v>55.0</v>
+        <v>0.0</v>
       </c>
       <c r="E54" s="4">
-        <v>20.0</v>
+        <v>0.0</v>
       </c>
       <c r="F54" s="2">
         <v>1.0</v>
@@ -5994,8 +6009,8 @@
       <c r="G54" s="2">
         <v>1.0</v>
       </c>
-      <c r="H54" s="2">
-        <v>0.0</v>
+      <c r="H54" s="4">
+        <v>1.0</v>
       </c>
       <c r="I54" s="2">
         <v>0.0</v>
@@ -6018,25 +6033,25 @@
       <c r="O54" s="2">
         <v>0.0</v>
       </c>
-      <c r="P54" s="4">
+      <c r="P54" s="2">
         <v>530.0</v>
       </c>
     </row>
     <row r="55" ht="14.25" customHeight="1">
-      <c r="A55" s="4" t="s">
+      <c r="A55" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="2" t="s">
         <v>139</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D55" s="4">
-        <v>95.0</v>
-      </c>
-      <c r="E55" s="4">
-        <v>28.0</v>
+        <v>5</v>
+      </c>
+      <c r="D55" s="2">
+        <v>0.0</v>
+      </c>
+      <c r="E55" s="2">
+        <v>0.0</v>
       </c>
       <c r="F55" s="2">
         <v>1.0</v>
@@ -6060,10 +6075,10 @@
         <v>0.0</v>
       </c>
       <c r="M55" s="2">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="N55" s="2">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O55" s="2">
         <v>0.0</v>
@@ -6072,56 +6087,7 @@
         <v>540.0</v>
       </c>
     </row>
-    <row r="56" ht="14.25" customHeight="1">
-      <c r="A56" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D56" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="E56" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="F56" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="G56" s="2">
-        <v>1.0</v>
-      </c>
-      <c r="H56" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="I56" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="J56" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="K56" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="L56" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="M56" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="N56" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="O56" s="2">
-        <v>0.0</v>
-      </c>
-      <c r="P56" s="2">
-        <v>550.0</v>
-      </c>
-    </row>
+    <row r="56" ht="14.25" customHeight="1"/>
     <row r="57" ht="14.25" customHeight="1"/>
     <row r="58" ht="14.25" customHeight="1"/>
     <row r="59" ht="14.25" customHeight="1"/>
@@ -6321,7 +6287,7 @@
     <row r="253" ht="14.25" customHeight="1"/>
     <row r="254" ht="14.25" customHeight="1"/>
     <row r="255" ht="14.25" customHeight="1"/>
-    <row r="256" ht="14.25" customHeight="1"/>
+    <row r="256" ht="15.75" customHeight="1"/>
     <row r="257" ht="15.75" customHeight="1"/>
     <row r="258" ht="15.75" customHeight="1"/>
     <row r="259" ht="15.75" customHeight="1"/>
@@ -7068,7 +7034,6 @@
     <row r="1000" ht="15.75" customHeight="1"/>
     <row r="1001" ht="15.75" customHeight="1"/>
     <row r="1002" ht="15.75" customHeight="1"/>
-    <row r="1003" ht="15.75" customHeight="1"/>
   </sheetData>
   <autoFilter ref="$A$1:$P$1"/>
   <printOptions/>
@@ -7105,7 +7070,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>4</v>
@@ -7113,10 +7078,10 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C2" s="2">
         <v>10.0</v>
@@ -7133,10 +7098,10 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C3" s="2">
         <v>10.0</v>
@@ -7153,10 +7118,10 @@
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C4" s="2">
         <v>10.0</v>
@@ -7173,10 +7138,10 @@
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C5" s="2">
         <v>10.0</v>
@@ -7193,10 +7158,10 @@
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C6" s="2">
         <v>10.0</v>
@@ -7213,10 +7178,10 @@
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C7" s="2">
         <v>10.0</v>
@@ -7233,10 +7198,10 @@
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C8" s="2">
         <v>15.0</v>
@@ -7253,10 +7218,10 @@
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C9" s="2">
         <v>10.0</v>
@@ -7273,10 +7238,10 @@
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C10" s="2">
         <v>10.0</v>
@@ -7293,10 +7258,10 @@
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C11" s="2">
         <v>5.0</v>
@@ -7313,10 +7278,10 @@
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C12" s="2">
         <v>5.0</v>
@@ -7333,10 +7298,10 @@
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C13" s="2">
         <v>5.0</v>
@@ -7353,10 +7318,10 @@
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C14" s="2">
         <v>5.0</v>
@@ -7373,10 +7338,10 @@
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C15" s="2">
         <v>5.0</v>
@@ -7393,10 +7358,10 @@
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C16" s="2">
         <v>10.0</v>
@@ -7413,10 +7378,10 @@
     </row>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C17" s="2">
         <v>10.0</v>
@@ -7433,10 +7398,10 @@
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C18" s="2">
         <v>10.0</v>
@@ -7453,10 +7418,10 @@
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C19" s="2">
         <v>10.0</v>
@@ -7573,10 +7538,10 @@
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C25" s="2">
         <v>10.0</v>
@@ -7593,10 +7558,10 @@
     </row>
     <row r="26" ht="14.25" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C26" s="2">
         <v>15.0</v>
@@ -7613,10 +7578,10 @@
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C27" s="2">
         <v>10.0</v>
@@ -7633,10 +7598,10 @@
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C28" s="2">
         <v>10.0</v>
@@ -7653,10 +7618,10 @@
     </row>
     <row r="29" ht="14.25" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C29" s="2">
         <v>5.0</v>
@@ -7673,10 +7638,10 @@
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C30" s="2">
         <v>5.0</v>
@@ -7693,10 +7658,10 @@
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C31" s="2">
         <v>35.0</v>
@@ -7713,10 +7678,10 @@
     </row>
     <row r="32" ht="14.25" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C32" s="2">
         <v>25.0</v>
@@ -7733,10 +7698,10 @@
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C33" s="2">
         <v>15.0</v>
@@ -7756,7 +7721,7 @@
         <v>80</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C34" s="2">
         <v>40.0</v>
@@ -7773,10 +7738,10 @@
     </row>
     <row r="35" ht="14.25" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C35" s="2">
         <v>35.0</v>
@@ -7793,10 +7758,10 @@
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C36" s="2">
         <v>15.0</v>
@@ -7813,10 +7778,10 @@
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C37" s="2">
         <v>7.0</v>
@@ -8833,39 +8798,39 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>208</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>211</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>213</v>
       </c>
       <c r="D2" s="2">
         <v>1.0</v>
@@ -8880,7 +8845,7 @@
         <v>5.0</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>7</v>
@@ -8894,13 +8859,13 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>215</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>217</v>
       </c>
       <c r="D3" s="2">
         <v>0.0</v>
@@ -8915,7 +8880,7 @@
         <v>15.0</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>7</v>
@@ -8929,13 +8894,13 @@
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D4" s="2">
         <v>1.0</v>
@@ -8950,7 +8915,7 @@
         <v>20.0</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>7</v>
@@ -8964,13 +8929,13 @@
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D5" s="2">
         <v>1.0</v>
@@ -8985,7 +8950,7 @@
         <v>25.0</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>7</v>
@@ -8999,13 +8964,13 @@
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D6" s="2">
         <v>0.0</v>
@@ -9020,7 +8985,7 @@
         <v>30.0</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>7</v>
@@ -9034,13 +8999,13 @@
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D7" s="2">
         <v>1.0</v>
@@ -9055,7 +9020,7 @@
         <v>35.0</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>7</v>
@@ -9069,13 +9034,13 @@
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D8" s="2">
         <v>1.0</v>
@@ -9090,7 +9055,7 @@
         <v>45.0</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>7</v>
@@ -9104,13 +9069,13 @@
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D9" s="2">
         <v>1.0</v>
@@ -9125,7 +9090,7 @@
         <v>50.0</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>7</v>
@@ -9139,13 +9104,13 @@
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D10" s="2">
         <v>1.0</v>
@@ -9160,7 +9125,7 @@
         <v>55.0</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>10</v>
@@ -9174,13 +9139,13 @@
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D11" s="2">
         <v>1.0</v>
@@ -9195,7 +9160,7 @@
         <v>60.0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>10</v>
@@ -9209,13 +9174,13 @@
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D12" s="2">
         <v>1.0</v>
@@ -9230,7 +9195,7 @@
         <v>65.0</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>10</v>
@@ -9244,13 +9209,13 @@
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D13" s="2">
         <v>1.0</v>
@@ -9265,7 +9230,7 @@
         <v>70.0</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>10</v>
@@ -9279,13 +9244,13 @@
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D14" s="2">
         <v>1.0</v>
@@ -9300,7 +9265,7 @@
         <v>80.0</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>10</v>
@@ -9314,13 +9279,13 @@
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D15" s="2">
         <v>1.0</v>
@@ -9335,7 +9300,7 @@
         <v>90.0</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>10</v>
@@ -9349,13 +9314,13 @@
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D16" s="2">
         <v>1.0</v>
@@ -9370,7 +9335,7 @@
         <v>100.0</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>10</v>
@@ -9384,13 +9349,13 @@
     </row>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D17" s="2">
         <v>1.0</v>
@@ -9405,7 +9370,7 @@
         <v>110.0</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>10</v>
@@ -9419,13 +9384,13 @@
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D18" s="2">
         <v>0.0</v>
@@ -9440,7 +9405,7 @@
         <v>120.0</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>10</v>
@@ -9454,13 +9419,13 @@
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D19" s="2">
         <v>0.0</v>
@@ -9475,7 +9440,7 @@
         <v>130.0</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>10</v>
@@ -9489,13 +9454,13 @@
     </row>
     <row r="20" ht="14.25" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D20" s="2">
         <v>1.0</v>
@@ -9510,7 +9475,7 @@
         <v>140.0</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>7</v>
@@ -9524,13 +9489,13 @@
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D21" s="2">
         <v>1.0</v>
@@ -9545,7 +9510,7 @@
         <v>150.0</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>7</v>
@@ -9559,13 +9524,13 @@
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D22" s="2">
         <v>1.0</v>
@@ -9580,7 +9545,7 @@
         <v>160.0</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>7</v>
@@ -9594,13 +9559,13 @@
     </row>
     <row r="23" ht="14.25" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D23" s="2">
         <v>0.0</v>
@@ -9615,7 +9580,7 @@
         <v>170.0</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>7</v>
@@ -9629,13 +9594,13 @@
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D24" s="2">
         <v>0.0</v>
@@ -9650,7 +9615,7 @@
         <v>180.0</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>7</v>
@@ -9664,13 +9629,13 @@
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D25" s="2">
         <v>1.0</v>
@@ -9685,7 +9650,7 @@
         <v>190.0</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>7</v>
@@ -9699,13 +9664,13 @@
     </row>
     <row r="26" ht="14.25" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D26" s="2">
         <v>0.0</v>
@@ -9720,7 +9685,7 @@
         <v>62.0</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>10</v>
@@ -9734,13 +9699,13 @@
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="5" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D27" s="5">
         <v>1.0</v>
@@ -9755,7 +9720,7 @@
         <v>200.0</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>7</v>
@@ -9767,7 +9732,41 @@
         <v>0.0</v>
       </c>
     </row>
-    <row r="28" ht="14.25" customHeight="1"/>
+    <row r="28" ht="14.25" customHeight="1">
+      <c r="A28" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D28" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E28" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F28" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="G28" s="5">
+        <v>210.0</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J28" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="K28" s="5">
+        <v>0.0</v>
+      </c>
+    </row>
     <row r="29" ht="14.25" customHeight="1"/>
     <row r="30" ht="14.25" customHeight="1"/>
     <row r="31" ht="14.25" customHeight="1"/>
@@ -9966,7 +9965,7 @@
     <row r="224" ht="14.25" customHeight="1"/>
     <row r="225" ht="14.25" customHeight="1"/>
     <row r="226" ht="14.25" customHeight="1"/>
-    <row r="227" ht="15.75" customHeight="1"/>
+    <row r="227" ht="14.25" customHeight="1"/>
     <row r="228" ht="15.75" customHeight="1"/>
     <row r="229" ht="15.75" customHeight="1"/>
     <row r="230" ht="15.75" customHeight="1"/>
@@ -10740,6 +10739,7 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <autoFilter ref="$A$1:$K$1"/>
   <printOptions/>
@@ -10794,7 +10794,7 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>268</v>
@@ -10820,7 +10820,7 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>271</v>
@@ -10846,7 +10846,7 @@
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>274</v>
@@ -10872,7 +10872,7 @@
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>277</v>
@@ -10898,7 +10898,7 @@
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>280</v>
@@ -10924,10 +10924,10 @@
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>283</v>
@@ -10945,15 +10945,15 @@
         <v>10.0</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>284</v>
@@ -10976,10 +10976,10 @@
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>286</v>
@@ -10997,12 +10997,12 @@
         <v>30.0</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>287</v>
@@ -11028,10 +11028,10 @@
     </row>
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>290</v>
@@ -11049,12 +11049,12 @@
         <v>50.0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>291</v>
@@ -11080,7 +11080,7 @@
     </row>
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>294</v>
@@ -11106,7 +11106,7 @@
     </row>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>297</v>
@@ -11132,7 +11132,7 @@
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>300</v>
@@ -11158,7 +11158,7 @@
     </row>
     <row r="16" ht="14.25" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>303</v>
@@ -11184,7 +11184,7 @@
     </row>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>306</v>
@@ -11210,10 +11210,10 @@
     </row>
     <row r="18" ht="14.25" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>309</v>
@@ -11231,12 +11231,12 @@
         <v>10.0</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>310</v>
@@ -11262,7 +11262,7 @@
     </row>
     <row r="20" ht="14.25" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>70</v>
@@ -11288,7 +11288,7 @@
     </row>
     <row r="21" ht="14.25" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>72</v>
@@ -11314,7 +11314,7 @@
     </row>
     <row r="22" ht="14.25" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>74</v>
@@ -11340,7 +11340,7 @@
     </row>
     <row r="23" ht="14.25" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>76</v>
@@ -11366,7 +11366,7 @@
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>321</v>
@@ -11392,7 +11392,7 @@
     </row>
     <row r="25" ht="14.25" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>324</v>
@@ -11418,7 +11418,7 @@
     </row>
     <row r="26" ht="14.25" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>327</v>
@@ -11444,7 +11444,7 @@
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>330</v>
@@ -11470,7 +11470,7 @@
     </row>
     <row r="28" ht="14.25" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>333</v>
@@ -11496,7 +11496,7 @@
     </row>
     <row r="29" ht="14.25" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>336</v>
@@ -11522,7 +11522,7 @@
     </row>
     <row r="30" ht="14.25" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>339</v>
@@ -11548,7 +11548,7 @@
     </row>
     <row r="31" ht="14.25" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>342</v>
@@ -11574,7 +11574,7 @@
     </row>
     <row r="32" ht="14.25" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>345</v>
@@ -11600,7 +11600,7 @@
     </row>
     <row r="33" ht="14.25" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>348</v>
@@ -11626,7 +11626,7 @@
     </row>
     <row r="34" ht="14.25" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>351</v>
@@ -11652,7 +11652,7 @@
     </row>
     <row r="35" ht="14.25" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>354</v>
@@ -11678,7 +11678,7 @@
     </row>
     <row r="36" ht="14.25" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>357</v>
@@ -11704,7 +11704,7 @@
     </row>
     <row r="37" ht="14.25" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>360</v>
@@ -11730,7 +11730,7 @@
     </row>
     <row r="38" ht="14.25" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>363</v>
@@ -11756,7 +11756,7 @@
     </row>
     <row r="39" ht="14.25" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>366</v>
@@ -11782,7 +11782,7 @@
     </row>
     <row r="40" ht="14.25" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>369</v>
@@ -11808,7 +11808,7 @@
     </row>
     <row r="41" ht="14.25" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>372</v>
@@ -11834,7 +11834,7 @@
     </row>
     <row r="42" ht="14.25" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>375</v>
@@ -11860,7 +11860,7 @@
     </row>
     <row r="43" ht="14.25" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>378</v>
@@ -11886,7 +11886,7 @@
     </row>
     <row r="44" ht="14.25" customHeight="1">
       <c r="A44" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>381</v>
@@ -11912,7 +11912,7 @@
     </row>
     <row r="45" ht="14.25" customHeight="1">
       <c r="A45" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>384</v>
@@ -11938,7 +11938,7 @@
     </row>
     <row r="46" ht="14.25" customHeight="1">
       <c r="A46" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>387</v>
@@ -11964,7 +11964,7 @@
     </row>
     <row r="47" ht="14.25" customHeight="1">
       <c r="A47" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>390</v>
@@ -11990,7 +11990,7 @@
     </row>
     <row r="48" ht="14.25" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>393</v>
@@ -12016,7 +12016,7 @@
     </row>
     <row r="49" ht="14.25" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>396</v>
@@ -12042,7 +12042,7 @@
     </row>
     <row r="50" ht="14.25" customHeight="1">
       <c r="A50" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>399</v>
@@ -12068,7 +12068,7 @@
     </row>
     <row r="51" ht="14.25" customHeight="1">
       <c r="A51" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>402</v>
@@ -12094,7 +12094,7 @@
     </row>
     <row r="52" ht="14.25" customHeight="1">
       <c r="A52" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>405</v>
@@ -12120,7 +12120,7 @@
     </row>
     <row r="53" ht="14.25" customHeight="1">
       <c r="A53" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>408</v>
@@ -12146,7 +12146,7 @@
     </row>
     <row r="54" ht="14.25" customHeight="1">
       <c r="A54" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>411</v>
@@ -12172,7 +12172,7 @@
     </row>
     <row r="55" ht="14.25" customHeight="1">
       <c r="A55" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>414</v>
@@ -12198,7 +12198,7 @@
     </row>
     <row r="56" ht="14.25" customHeight="1">
       <c r="A56" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>417</v>
@@ -12224,7 +12224,7 @@
     </row>
     <row r="57" ht="14.25" customHeight="1">
       <c r="A57" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>420</v>
@@ -12250,7 +12250,7 @@
     </row>
     <row r="58" ht="14.25" customHeight="1">
       <c r="A58" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>423</v>
@@ -12276,7 +12276,7 @@
     </row>
     <row r="59" ht="14.25" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B59" s="4" t="s">
         <v>426</v>
@@ -12302,7 +12302,7 @@
     </row>
     <row r="60" ht="14.25" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>429</v>
@@ -12328,7 +12328,7 @@
     </row>
     <row r="61" ht="14.25" customHeight="1">
       <c r="A61" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>432</v>
@@ -12354,7 +12354,7 @@
     </row>
     <row r="62" ht="14.25" customHeight="1">
       <c r="A62" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>435</v>
@@ -12380,7 +12380,7 @@
     </row>
     <row r="63" ht="14.25" customHeight="1">
       <c r="A63" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>437</v>
@@ -12406,7 +12406,7 @@
     </row>
     <row r="64" ht="14.25" customHeight="1">
       <c r="A64" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>439</v>
@@ -12432,7 +12432,7 @@
     </row>
     <row r="65" ht="14.25" customHeight="1">
       <c r="A65" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>441</v>
@@ -12458,7 +12458,7 @@
     </row>
     <row r="66" ht="14.25" customHeight="1">
       <c r="A66" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>443</v>
@@ -12484,7 +12484,7 @@
     </row>
     <row r="67" ht="14.25" customHeight="1">
       <c r="A67" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>445</v>
@@ -12510,7 +12510,7 @@
     </row>
     <row r="68" ht="14.25" customHeight="1">
       <c r="A68" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>447</v>
@@ -12536,7 +12536,7 @@
     </row>
     <row r="69" ht="14.25" customHeight="1">
       <c r="A69" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>449</v>
@@ -12562,7 +12562,7 @@
     </row>
     <row r="70" ht="14.25" customHeight="1">
       <c r="A70" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>451</v>
@@ -12588,7 +12588,7 @@
     </row>
     <row r="71" ht="14.25" customHeight="1">
       <c r="A71" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>453</v>
@@ -12614,7 +12614,7 @@
     </row>
     <row r="72" ht="14.25" customHeight="1">
       <c r="A72" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>455</v>
@@ -12640,13 +12640,13 @@
     </row>
     <row r="73" ht="14.25" customHeight="1">
       <c r="A73" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D73" s="2">
         <v>0.0</v>
@@ -12661,12 +12661,12 @@
         <v>10.0</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="74" ht="14.25" customHeight="1">
       <c r="A74" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>80</v>
@@ -12692,10 +12692,10 @@
     </row>
     <row r="75" ht="14.25" customHeight="1">
       <c r="A75" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C75" s="2" t="s">
         <v>459</v>
@@ -12718,10 +12718,10 @@
     </row>
     <row r="76" ht="14.25" customHeight="1">
       <c r="A76" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>461</v>
@@ -12744,10 +12744,10 @@
     </row>
     <row r="77" ht="14.25" customHeight="1">
       <c r="A77" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>463</v>
@@ -12770,10 +12770,10 @@
     </row>
     <row r="78" ht="14.25" customHeight="1">
       <c r="A78" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>465</v>
@@ -12796,10 +12796,10 @@
     </row>
     <row r="79" ht="14.25" customHeight="1">
       <c r="A79" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>467</v>
@@ -12822,7 +12822,7 @@
     </row>
     <row r="80" ht="14.25" customHeight="1">
       <c r="A80" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>469</v>
@@ -12848,7 +12848,7 @@
     </row>
     <row r="81" ht="14.25" customHeight="1">
       <c r="A81" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>472</v>
@@ -12874,7 +12874,7 @@
     </row>
     <row r="82" ht="14.25" customHeight="1">
       <c r="A82" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>475</v>
@@ -12900,7 +12900,7 @@
     </row>
     <row r="83" ht="14.25" customHeight="1">
       <c r="A83" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>478</v>
@@ -12926,7 +12926,7 @@
     </row>
     <row r="84" ht="14.25" customHeight="1">
       <c r="A84" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>480</v>
@@ -12952,7 +12952,7 @@
     </row>
     <row r="85" ht="14.25" customHeight="1">
       <c r="A85" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>482</v>
@@ -12978,7 +12978,7 @@
     </row>
     <row r="86" ht="14.25" customHeight="1">
       <c r="A86" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>484</v>
@@ -13004,7 +13004,7 @@
     </row>
     <row r="87" ht="14.25" customHeight="1">
       <c r="A87" s="2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>486</v>
@@ -13030,13 +13030,13 @@
     </row>
     <row r="88" ht="14.25" customHeight="1">
       <c r="A88" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D88" s="2">
         <v>0.0</v>
@@ -13051,12 +13051,12 @@
         <v>10.0</v>
       </c>
       <c r="H88" s="2" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="89" ht="14.25" customHeight="1">
       <c r="A89" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>488</v>
@@ -13082,7 +13082,7 @@
     </row>
     <row r="90" ht="14.25" customHeight="1">
       <c r="A90" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B90" s="3" t="s">
         <v>491</v>
@@ -13108,7 +13108,7 @@
     </row>
     <row r="91" ht="14.25" customHeight="1">
       <c r="A91" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B91" s="3" t="s">
         <v>494</v>
@@ -13134,7 +13134,7 @@
     </row>
     <row r="92" ht="14.25" customHeight="1">
       <c r="A92" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B92" s="3" t="s">
         <v>497</v>
@@ -13160,7 +13160,7 @@
     </row>
     <row r="93" ht="14.25" customHeight="1">
       <c r="A93" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B93" s="3" t="s">
         <v>500</v>
@@ -13186,7 +13186,7 @@
     </row>
     <row r="94" ht="14.25" customHeight="1">
       <c r="A94" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>503</v>
@@ -13212,7 +13212,7 @@
     </row>
     <row r="95" ht="14.25" customHeight="1">
       <c r="A95" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>110</v>
@@ -13238,7 +13238,7 @@
     </row>
     <row r="96" ht="14.25" customHeight="1">
       <c r="A96" s="5" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>507</v>
@@ -13247,10 +13247,10 @@
         <v>508</v>
       </c>
       <c r="D96" s="5">
-        <v>0.0</v>
+        <v>55.0</v>
       </c>
       <c r="E96" s="5">
-        <v>0.0</v>
+        <v>20.0</v>
       </c>
       <c r="F96" s="5">
         <v>1.0</v>
@@ -13264,7 +13264,7 @@
     </row>
     <row r="97" ht="14.25" customHeight="1">
       <c r="A97" s="5" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>510</v>
@@ -13273,10 +13273,10 @@
         <v>511</v>
       </c>
       <c r="D97" s="5">
-        <v>0.0</v>
+        <v>95.0</v>
       </c>
       <c r="E97" s="5">
-        <v>0.0</v>
+        <v>28.0</v>
       </c>
       <c r="F97" s="5">
         <v>1.0</v>
@@ -13308,7 +13308,7 @@
         <v>1.0</v>
       </c>
       <c r="G98" s="5">
-        <v>30.0</v>
+        <v>10.0</v>
       </c>
       <c r="H98" s="5" t="s">
         <v>515</v>
@@ -13334,14 +13334,64 @@
         <v>1.0</v>
       </c>
       <c r="G99" s="5">
-        <v>40.0</v>
+        <v>20.0</v>
       </c>
       <c r="H99" s="5" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="100" ht="14.25" customHeight="1"/>
-    <row r="101" ht="14.25" customHeight="1"/>
+    <row r="100" ht="14.25" customHeight="1">
+      <c r="A100" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="C100" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="D100" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E100" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F100" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="G100" s="5">
+        <v>30.0</v>
+      </c>
+      <c r="H100" s="5" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="101" ht="14.25" customHeight="1">
+      <c r="A101" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="B101" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="C101" s="5" t="s">
+        <v>523</v>
+      </c>
+      <c r="D101" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E101" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="F101" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="G101" s="5">
+        <v>40.0</v>
+      </c>
+      <c r="H101" s="5" t="s">
+        <v>524</v>
+      </c>
+    </row>
     <row r="102" ht="14.25" customHeight="1"/>
     <row r="103" ht="14.25" customHeight="1"/>
     <row r="104" ht="14.25" customHeight="1"/>
@@ -13536,8 +13586,8 @@
     <row r="293" ht="14.25" customHeight="1"/>
     <row r="294" ht="14.25" customHeight="1"/>
     <row r="295" ht="14.25" customHeight="1"/>
-    <row r="296" ht="15.75" customHeight="1"/>
-    <row r="297" ht="15.75" customHeight="1"/>
+    <row r="296" ht="14.25" customHeight="1"/>
+    <row r="297" ht="14.25" customHeight="1"/>
     <row r="298" ht="15.75" customHeight="1"/>
     <row r="299" ht="15.75" customHeight="1"/>
     <row r="300" ht="15.75" customHeight="1"/>
@@ -14243,6 +14293,8 @@
     <row r="1000" ht="15.75" customHeight="1"/>
     <row r="1001" ht="15.75" customHeight="1"/>
     <row r="1002" ht="15.75" customHeight="1"/>
+    <row r="1003" ht="15.75" customHeight="1"/>
+    <row r="1004" ht="15.75" customHeight="1"/>
   </sheetData>
   <autoFilter ref="$A$1:$H$1"/>
   <printOptions/>
@@ -14270,22 +14322,22 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>266</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>206</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>3</v>
@@ -14296,7 +14348,7 @@
         <v>38</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C2" s="2">
         <v>1.0</v>
@@ -14305,7 +14357,7 @@
         <v>0.0</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F2" s="2">
         <v>5.0</v>
@@ -14319,7 +14371,7 @@
         <v>42</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C3" s="2">
         <v>1.0</v>
@@ -14328,7 +14380,7 @@
         <v>0.0</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F3" s="2">
         <v>5.0</v>
@@ -14342,7 +14394,7 @@
         <v>44</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C4" s="2">
         <v>1.0</v>
@@ -14351,7 +14403,7 @@
         <v>0.0</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F4" s="2">
         <v>5.0</v>
@@ -14365,7 +14417,7 @@
         <v>46</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C5" s="2">
         <v>0.0</v>
@@ -14374,7 +14426,7 @@
         <v>1.0</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F5" s="2">
         <v>5.0</v>
@@ -14388,7 +14440,7 @@
         <v>48</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C6" s="2">
         <v>1.0</v>
@@ -14397,7 +14449,7 @@
         <v>0.0</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F6" s="2">
         <v>5.0</v>
@@ -14411,7 +14463,7 @@
         <v>32</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C7" s="2">
         <v>1.0</v>
@@ -14420,7 +14472,7 @@
         <v>0.0</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F7" s="2">
         <v>5.0</v>
@@ -14434,7 +14486,7 @@
         <v>32</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C8" s="2">
         <v>0.0</v>
@@ -14443,7 +14495,7 @@
         <v>1.0</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F8" s="2">
         <v>10.0</v>
@@ -14457,7 +14509,7 @@
         <v>34</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C9" s="2">
         <v>1.0</v>
@@ -14466,7 +14518,7 @@
         <v>0.0</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F9" s="2">
         <v>5.0</v>
@@ -14480,7 +14532,7 @@
         <v>34</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C10" s="2">
         <v>0.0</v>
@@ -14489,7 +14541,7 @@
         <v>1.0</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F10" s="2">
         <v>10.0</v>
@@ -14503,7 +14555,7 @@
         <v>58</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C11" s="2">
         <v>1.0</v>
@@ -14512,7 +14564,7 @@
         <v>0.0</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F11" s="2">
         <v>5.0</v>
@@ -14526,7 +14578,7 @@
         <v>102</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C12" s="2">
         <v>1.0</v>
@@ -14535,7 +14587,7 @@
         <v>0.0</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F12" s="2">
         <v>5.0</v>
@@ -14549,7 +14601,7 @@
         <v>104</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C13" s="2">
         <v>1.0</v>
@@ -14558,7 +14610,7 @@
         <v>0.0</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F13" s="2">
         <v>5.0</v>
@@ -14572,7 +14624,7 @@
         <v>36</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C14" s="2">
         <v>1.0</v>
@@ -14581,7 +14633,7 @@
         <v>0.0</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F14" s="2">
         <v>5.0</v>
@@ -14595,7 +14647,7 @@
         <v>36</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C15" s="2">
         <v>1.0</v>
@@ -14604,7 +14656,7 @@
         <v>0.0</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F15" s="2">
         <v>10.0</v>
@@ -14618,7 +14670,7 @@
         <v>112</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C16" s="2">
         <v>1.0</v>
@@ -14627,7 +14679,7 @@
         <v>0.0</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F16" s="2">
         <v>5.0</v>
@@ -14641,7 +14693,7 @@
         <v>110</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C17" s="2">
         <v>1.0</v>
@@ -14650,7 +14702,7 @@
         <v>0.0</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F17" s="2">
         <v>5.0</v>
@@ -14664,7 +14716,7 @@
         <v>114</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C18" s="2">
         <v>1.0</v>
@@ -14673,7 +14725,7 @@
         <v>0.0</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F18" s="2">
         <v>5.0</v>
@@ -14687,7 +14739,7 @@
         <v>116</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C19" s="2">
         <v>1.0</v>
@@ -14696,7 +14748,7 @@
         <v>0.0</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F19" s="2">
         <v>5.0</v>
@@ -14710,7 +14762,7 @@
         <v>116</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C20" s="2">
         <v>1.0</v>
@@ -14719,7 +14771,7 @@
         <v>0.0</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F20" s="2">
         <v>10.0</v>
@@ -14733,7 +14785,7 @@
         <v>118</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C21" s="2">
         <v>1.0</v>
@@ -14742,7 +14794,7 @@
         <v>0.0</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F21" s="2">
         <v>5.0</v>
@@ -14756,7 +14808,7 @@
         <v>118</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C22" s="2">
         <v>1.0</v>
@@ -14765,7 +14817,7 @@
         <v>0.0</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F22" s="2">
         <v>10.0</v>
@@ -14779,7 +14831,7 @@
         <v>120</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C23" s="2">
         <v>1.0</v>
@@ -14788,7 +14840,7 @@
         <v>0.0</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F23" s="2">
         <v>5.0</v>
@@ -14802,7 +14854,7 @@
         <v>122</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C24" s="2">
         <v>1.0</v>
@@ -14811,7 +14863,7 @@
         <v>0.0</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F24" s="2">
         <v>5.0</v>
@@ -14825,7 +14877,7 @@
         <v>124</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C25" s="2">
         <v>1.0</v>
@@ -14834,7 +14886,7 @@
         <v>0.0</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F25" s="2">
         <v>5.0</v>
@@ -14848,7 +14900,7 @@
         <v>124</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C26" s="2">
         <v>1.0</v>
@@ -14857,7 +14909,7 @@
         <v>0.0</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F26" s="2">
         <v>10.0</v>
@@ -14871,7 +14923,7 @@
         <v>124</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C27" s="2">
         <v>1.0</v>
@@ -14880,7 +14932,7 @@
         <v>0.0</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F27" s="2">
         <v>15.0</v>
@@ -14894,7 +14946,7 @@
         <v>124</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C28" s="2">
         <v>0.0</v>
@@ -14903,7 +14955,7 @@
         <v>0.0</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F28" s="2">
         <v>20.0</v>
@@ -14917,7 +14969,7 @@
         <v>126</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C29" s="2">
         <v>0.0</v>
@@ -14926,7 +14978,7 @@
         <v>0.0</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F29" s="2">
         <v>5.0</v>
@@ -14940,7 +14992,7 @@
         <v>70</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C30" s="2">
         <v>1.0</v>
@@ -14949,7 +15001,7 @@
         <v>0.0</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F30" s="2">
         <v>5.0</v>
@@ -14963,7 +15015,7 @@
         <v>72</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C31" s="2">
         <v>1.0</v>
@@ -14972,7 +15024,7 @@
         <v>0.0</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F31" s="2">
         <v>10.0</v>
@@ -14986,7 +15038,7 @@
         <v>74</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C32" s="2">
         <v>1.0</v>
@@ -14995,7 +15047,7 @@
         <v>0.0</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F32" s="2">
         <v>15.0</v>
@@ -15009,7 +15061,7 @@
         <v>76</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C33" s="2">
         <v>1.0</v>
@@ -15018,7 +15070,7 @@
         <v>0.0</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F33" s="2">
         <v>20.0</v>
@@ -15032,7 +15084,7 @@
         <v>78</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C34" s="2">
         <v>1.0</v>
@@ -15041,7 +15093,7 @@
         <v>0.0</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F34" s="2">
         <v>25.0</v>
@@ -15055,7 +15107,7 @@
         <v>80</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C35" s="2">
         <v>1.0</v>
@@ -15064,7 +15116,7 @@
         <v>0.0</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F35" s="2">
         <v>30.0</v>
@@ -15078,7 +15130,7 @@
         <v>40</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C36" s="2">
         <v>1.0</v>
@@ -15087,7 +15139,7 @@
         <v>0.0</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F36" s="2">
         <v>5.0</v>
@@ -15101,7 +15153,7 @@
         <v>60</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C37" s="2">
         <v>1.0</v>
@@ -15110,7 +15162,7 @@
         <v>0.0</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F37" s="2">
         <v>5.0</v>
@@ -15119,8 +15171,52 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="38" ht="14.25" customHeight="1"/>
-    <row r="39" ht="14.25" customHeight="1"/>
+    <row r="38" ht="14.25" customHeight="1">
+      <c r="A38" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="C38" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="D38" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="F38" s="5">
+        <v>5.0</v>
+      </c>
+      <c r="G38" s="5">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="39" ht="14.25" customHeight="1">
+      <c r="A39" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="C39" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="D39" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="F39" s="5">
+        <v>10.0</v>
+      </c>
+      <c r="G39" s="5">
+        <v>1.0</v>
+      </c>
+    </row>
     <row r="40" ht="14.25" customHeight="1"/>
     <row r="41" ht="14.25" customHeight="1"/>
     <row r="42" ht="14.25" customHeight="1"/>
@@ -16109,19 +16205,19 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>4</v>
@@ -16135,13 +16231,13 @@
         <v>32</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="E2" s="2">
         <v>1.0</v>
@@ -16158,13 +16254,13 @@
         <v>34</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="E3" s="2">
         <v>1.0</v>
@@ -16181,13 +16277,13 @@
         <v>36</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="E4" s="2">
         <v>1.0</v>
@@ -16204,13 +16300,13 @@
         <v>38</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E5" s="2">
         <v>1.0</v>
@@ -16227,13 +16323,13 @@
         <v>40</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="E6" s="2">
         <v>1.0</v>
@@ -16250,13 +16346,13 @@
         <v>42</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="E7" s="2">
         <v>1.0</v>
@@ -16273,13 +16369,13 @@
         <v>44</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="E8" s="2">
         <v>1.0</v>
@@ -16296,13 +16392,13 @@
         <v>46</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="E9" s="2">
         <v>1.0</v>
@@ -16319,13 +16415,13 @@
         <v>48</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="E10" s="2">
         <v>1.0</v>
@@ -16342,13 +16438,13 @@
         <v>50</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="E11" s="2">
         <v>1.0</v>
@@ -16365,13 +16461,13 @@
         <v>52</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="E12" s="2">
         <v>1.0</v>
@@ -16388,13 +16484,13 @@
         <v>54</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="E13" s="2">
         <v>1.0</v>
@@ -16411,13 +16507,13 @@
         <v>56</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="E14" s="2">
         <v>1.0</v>
@@ -16434,13 +16530,13 @@
         <v>58</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="E15" s="2">
         <v>1.0</v>
@@ -16457,13 +16553,13 @@
         <v>60</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="E16" s="2">
         <v>1.0</v>
@@ -16480,13 +16576,13 @@
         <v>62</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="E17" s="2">
         <v>1.0</v>
@@ -16503,13 +16599,13 @@
         <v>64</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="E18" s="2">
         <v>1.0</v>
@@ -16526,13 +16622,13 @@
         <v>66</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="E19" s="2">
         <v>1.0</v>
@@ -16549,13 +16645,13 @@
         <v>68</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="E20" s="2">
         <v>1.0</v>
@@ -16572,13 +16668,13 @@
         <v>70</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="E21" s="2">
         <v>1.0</v>
@@ -16595,13 +16691,13 @@
         <v>72</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="E22" s="2">
         <v>1.0</v>
@@ -16618,13 +16714,13 @@
         <v>74</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="E23" s="2">
         <v>1.0</v>
@@ -16641,13 +16737,13 @@
         <v>76</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="E24" s="2">
         <v>1.0</v>
@@ -16664,13 +16760,13 @@
         <v>78</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="E25" s="2">
         <v>1.0</v>
@@ -16687,13 +16783,13 @@
         <v>80</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="E26" s="2">
         <v>1.0</v>
@@ -16710,13 +16806,13 @@
         <v>82</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="E27" s="2">
         <v>1.0</v>
@@ -16733,13 +16829,13 @@
         <v>84</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="E28" s="2">
         <v>1.0</v>
@@ -16756,13 +16852,13 @@
         <v>86</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="E29" s="2">
         <v>1.0</v>
@@ -16779,13 +16875,13 @@
         <v>88</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="E30" s="2">
         <v>1.0</v>
@@ -16802,13 +16898,13 @@
         <v>90</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="E31" s="2">
         <v>1.0</v>
@@ -16825,13 +16921,13 @@
         <v>92</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="E32" s="2">
         <v>1.0</v>
@@ -16848,13 +16944,13 @@
         <v>94</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="E33" s="2">
         <v>1.0</v>
@@ -16871,13 +16967,13 @@
         <v>96</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="E34" s="2">
         <v>1.0</v>
@@ -16894,13 +16990,13 @@
         <v>98</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="E35" s="2">
         <v>1.0</v>
@@ -16917,13 +17013,13 @@
         <v>100</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="E36" s="2">
         <v>1.0</v>
@@ -16940,13 +17036,13 @@
         <v>102</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="E37" s="2">
         <v>1.0</v>
@@ -16963,13 +17059,13 @@
         <v>104</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="E38" s="2">
         <v>1.0</v>
@@ -16986,13 +17082,13 @@
         <v>106</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="E39" s="4">
         <v>1.0</v>
@@ -17009,13 +17105,13 @@
         <v>108</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="E40" s="2">
         <v>1.0</v>
@@ -17032,13 +17128,13 @@
         <v>110</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="E41" s="2">
         <v>1.0</v>
@@ -17055,13 +17151,13 @@
         <v>112</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="E42" s="2">
         <v>1.0</v>
@@ -17078,13 +17174,13 @@
         <v>114</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="E43" s="2">
         <v>1.0</v>
@@ -17101,13 +17197,13 @@
         <v>116</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="E44" s="2">
         <v>1.0</v>
@@ -17124,13 +17220,13 @@
         <v>118</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="E45" s="2">
         <v>1.0</v>
@@ -17147,13 +17243,13 @@
         <v>120</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="E46" s="2">
         <v>1.0</v>
@@ -17170,13 +17266,13 @@
         <v>122</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="E47" s="2">
         <v>1.0</v>
@@ -17193,13 +17289,13 @@
         <v>124</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="E48" s="2">
         <v>1.0</v>
@@ -17216,13 +17312,13 @@
         <v>126</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="E49" s="2">
         <v>1.0</v>
@@ -17239,13 +17335,13 @@
         <v>128</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
       <c r="E50" s="2">
         <v>1.0</v>
@@ -17262,13 +17358,13 @@
         <v>130</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="E51" s="2">
         <v>1.0</v>
@@ -17285,13 +17381,13 @@
         <v>132</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="E52" s="2">
         <v>1.0</v>
@@ -17308,13 +17404,13 @@
         <v>134</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
       <c r="E53" s="2">
         <v>1.0</v>
@@ -17331,13 +17427,13 @@
         <v>136</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="E54" s="5">
         <v>1.0</v>
@@ -17349,29 +17445,7 @@
         <v>1.0</v>
       </c>
     </row>
-    <row r="55" ht="14.25" customHeight="1">
-      <c r="A55" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="B55" s="5" t="s">
-        <v>526</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D55" s="5" t="s">
-        <v>579</v>
-      </c>
-      <c r="E55" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="F55" s="2">
-        <v>540.0</v>
-      </c>
-      <c r="G55" s="5">
-        <v>1.0</v>
-      </c>
-    </row>
+    <row r="55" ht="14.25" customHeight="1"/>
     <row r="56" ht="14.25" customHeight="1"/>
     <row r="57" ht="14.25" customHeight="1"/>
     <row r="58" ht="14.25" customHeight="1"/>
@@ -17569,7 +17643,7 @@
     <row r="250" ht="14.25" customHeight="1"/>
     <row r="251" ht="14.25" customHeight="1"/>
     <row r="252" ht="14.25" customHeight="1"/>
-    <row r="253" ht="14.25" customHeight="1"/>
+    <row r="253" ht="15.75" customHeight="1"/>
     <row r="254" ht="15.75" customHeight="1"/>
     <row r="255" ht="15.75" customHeight="1"/>
     <row r="256" ht="15.75" customHeight="1"/>
@@ -18317,7 +18391,6 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
-    <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <autoFilter ref="$A$1:$G$1"/>
   <printOptions/>
@@ -18353,7 +18426,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
@@ -18364,13 +18437,13 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>581</v>
+        <v>586</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="E2" s="2">
         <v>1.0</v>
@@ -18381,13 +18454,13 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>584</v>
+        <v>589</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>582</v>
+        <v>587</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>585</v>
+        <v>590</v>
       </c>
       <c r="E3" s="2">
         <v>1.0</v>
@@ -19416,50 +19489,50 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="6" t="s">
-        <v>586</v>
+        <v>591</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>587</v>
+        <v>592</v>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="7" t="s">
-        <v>588</v>
+        <v>593</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>589</v>
+        <v>594</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="7" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>591</v>
+        <v>596</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>592</v>
+        <v>597</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>593</v>
+        <v>598</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="7" t="s">
-        <v>594</v>
+        <v>599</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>595</v>
+        <v>600</v>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="7" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
@@ -19467,31 +19540,31 @@
         <v>37</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="7" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="7" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>601</v>
+        <v>606</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="7" t="s">
-        <v>602</v>
+        <v>607</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">

</xml_diff>